<commit_message>
MIN instead of IF < when applying fairshare
</commit_message>
<xml_diff>
--- a/fairshare.xlsx
+++ b/fairshare.xlsx
@@ -336,39 +336,6 @@
                 <xdr:colOff>47</xdr:colOff>
                 <xdr:row>19</xdr:row>
                 <xdr:rowOff>13</xdr:rowOff>
-              </xdr:to>
-            </anchor>
-          </commentPr>
-        </mc:Choice>
-        <mc:Fallback/>
-      </mc:AlternateContent>
-    </comment>
-    <comment ref="G1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Ergebnis: Falls möglich, ist Dein Glas voll. Falls nicht, bekommst Du immerhin nicht weniger als irgendjemand sonst.</t>
-        </r>
-      </text>
-      <mc:AlternateContent>
-        <mc:Choice Requires="v2">
-          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
-            <anchor moveWithCells="false" sizeWithCells="false">
-              <xdr:from>
-                <xdr:col>7</xdr:col>
-                <xdr:colOff>23</xdr:colOff>
-                <xdr:row>0</xdr:row>
-                <xdr:rowOff>0</xdr:rowOff>
-              </xdr:from>
-              <xdr:to>
-                <xdr:col>8</xdr:col>
-                <xdr:colOff>47</xdr:colOff>
-                <xdr:row>7</xdr:row>
-                <xdr:rowOff>8</xdr:rowOff>
               </xdr:to>
             </anchor>
           </commentPr>
@@ -1507,7 +1474,7 @@
         <v>1</v>
       </c>
       <c r="G1" s="5" t="n">
-        <f aca="false">IF(B1&lt;F1,B1,fairshare)</f>
+        <f aca="false">MIN(B1,fairshare)</f>
         <v>0.5</v>
       </c>
     </row>
@@ -1535,7 +1502,7 @@
         <v>1.1</v>
       </c>
       <c r="G2" s="7" t="n">
-        <f aca="false">IF(B2&lt;F2,B2,fairshare)</f>
+        <f aca="false">MIN(B2,fairshare)</f>
         <v>0.7</v>
       </c>
       <c r="I2" s="8" t="s">
@@ -1569,7 +1536,7 @@
         <v>1.2</v>
       </c>
       <c r="G3" s="7" t="n">
-        <f aca="false">IF(B3&lt;F3,B3,fairshare)</f>
+        <f aca="false">MIN(B3,fairshare)</f>
         <v>1.2</v>
       </c>
       <c r="I3" s="8"/>
@@ -1601,7 +1568,7 @@
         <v>1.2</v>
       </c>
       <c r="G4" s="7" t="n">
-        <f aca="false">IF(B4&lt;F4,B4,fairshare)</f>
+        <f aca="false">MIN(B4,fairshare)</f>
         <v>1.2</v>
       </c>
       <c r="I4" s="8"/>
@@ -1633,7 +1600,7 @@
         <v>1.15</v>
       </c>
       <c r="G5" s="7" t="n">
-        <f aca="false">IF(B5&lt;F5,B5,fairshare)</f>
+        <f aca="false">MIN(B5,fairshare)</f>
         <v>1.2</v>
       </c>
       <c r="I5" s="8"/>
@@ -1665,7 +1632,7 @@
         <v>0.5</v>
       </c>
       <c r="G6" s="10" t="n">
-        <f aca="false">IF(B6&lt;F6,B6,fairshare)</f>
+        <f aca="false">MIN(B6,fairshare)</f>
         <v>1.2</v>
       </c>
     </row>

</xml_diff>